<commit_message>
Lower default allotment push concurrency from 8 to 4, update runtime data snapshot
Reduces the default max_workers for the PMS allotment batch push across
all entry points (Fast API Pipeline, bulk push route, PMS API test page)
as a safety margin against the transient PMS-side timeouts/errors seen
under 8 concurrent requests. Also commits the latest pipeline run's
output to backend/app/scraper/data/.
</commit_message>
<xml_diff>
--- a/backend/app/scraper/data/cm_upload.xlsx
+++ b/backend/app/scraper/data/cm_upload.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <x:si>
-    <x:t>The Anvaya Beach Resorts Bali - Saturday, September 26, 2026 2:17:29 PM</x:t>
+    <x:t>The Anvaya Beach Resorts Bali - Saturday, September 26, 2026 3:11:59 PM</x:t>
   </x:si>
   <x:si>
     <x:t>Deluxe Room</x:t>
@@ -813,19 +813,19 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G2" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H2" s="3" t="n">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="I2" s="3" t="n">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="J2" s="3" t="n">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="K2" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L2" s="3" t="n">
         <x:v>0</x:v>
@@ -1059,25 +1059,25 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="CK2" s="3" t="n">
-        <x:v>32</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="CL2" s="3" t="n">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="CM2" s="3" t="n">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="CN2" s="3" t="n">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="CO2" s="3" t="n">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="CP2" s="3" t="n">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="CQ2" s="3" t="n">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="CR2" s="3" t="n">
         <x:v>30</x:v>
@@ -1809,7 +1809,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z6" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AA6" s="3" t="n">
         <x:v>0</x:v>
@@ -1854,7 +1854,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="AO6" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AP6" s="3" t="n">
         <x:v>2</x:v>
@@ -1947,7 +1947,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="BT6" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="BU6" s="3" t="n">
         <x:v>5</x:v>
@@ -2682,7 +2682,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="D10" s="3" t="n">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E10" s="3" t="n">
         <x:v>0</x:v>
@@ -2694,13 +2694,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H10" s="3" t="n">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="I10" s="3" t="n">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="J10" s="3" t="n">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="K10" s="3" t="n">
         <x:v>30</x:v>
@@ -3672,10 +3672,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="U14" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V14" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="W14" s="3" t="s">
         <x:v>3</x:v>
@@ -3756,7 +3756,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AW14" s="3" t="n">
-        <x:v>10</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AX14" s="3" t="n">
         <x:v>10</x:v>
@@ -3894,7 +3894,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="CQ14" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="CR14" s="3" t="n">
         <x:v>5</x:v>
@@ -5700,13 +5700,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="BS22" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="BT22" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="BU22" s="3" t="n">
         <x:v>4</x:v>
-      </x:c>
-      <x:c r="BT22" s="3" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="BU22" s="3" t="n">
-        <x:v>3</x:v>
       </x:c>
       <x:c r="BV22" s="3" t="n">
         <x:v>3</x:v>
@@ -6498,7 +6498,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="X26" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="Y26" s="3" t="n">
         <x:v>1</x:v>
@@ -7434,7 +7434,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="W30" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="X30" s="3" t="n">
         <x:v>0</x:v>
@@ -8367,37 +8367,37 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="U34" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V34" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="W34" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="X34" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="Y34" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Z34" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="AA34" s="3" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="Z34" s="3" t="n">
+      <x:c r="AB34" s="3" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="AA34" s="3" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="AB34" s="3" t="n">
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="AC34" s="3" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AD34" s="3" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AE34" s="3" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="AF34" s="3" t="n">
         <x:v>6</x:v>
@@ -8460,7 +8460,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AZ34" s="3" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="BA34" s="3" t="n">
         <x:v>3</x:v>
@@ -8610,13 +8610,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="CX34" s="3" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="CY34" s="3" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="CZ34" s="3" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:104">

</xml_diff>